<commit_message>
game: add novice crafting choices and preview growth rewards
Co-Authored-By: Codex <noreply@openai.com>
</commit_message>
<xml_diff>
--- a/Assets/@Resources/Data/Excel/EquipEnhanceData.xlsx
+++ b/Assets/@Resources/Data/Excel/EquipEnhanceData.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H543"/>
+  <dimension ref="A1:H561"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14582,6 +14582,474 @@
         <v>37</v>
       </c>
     </row>
+    <row r="544">
+      <c r="A544" t="n">
+        <v>541</v>
+      </c>
+      <c r="B544" t="n">
+        <v>30061</v>
+      </c>
+      <c r="C544" t="n">
+        <v>1</v>
+      </c>
+      <c r="D544" t="n">
+        <v>9</v>
+      </c>
+      <c r="E544" t="n">
+        <v>0</v>
+      </c>
+      <c r="F544" t="n">
+        <v>0</v>
+      </c>
+      <c r="G544" t="n">
+        <v>11001</v>
+      </c>
+      <c r="H544" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="545">
+      <c r="A545" t="n">
+        <v>542</v>
+      </c>
+      <c r="B545" t="n">
+        <v>30061</v>
+      </c>
+      <c r="C545" t="n">
+        <v>2</v>
+      </c>
+      <c r="D545" t="n">
+        <v>9</v>
+      </c>
+      <c r="E545" t="n">
+        <v>0</v>
+      </c>
+      <c r="F545" t="n">
+        <v>0</v>
+      </c>
+      <c r="G545" t="n">
+        <v>11001</v>
+      </c>
+      <c r="H545" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="546">
+      <c r="A546" t="n">
+        <v>543</v>
+      </c>
+      <c r="B546" t="n">
+        <v>30061</v>
+      </c>
+      <c r="C546" t="n">
+        <v>3</v>
+      </c>
+      <c r="D546" t="n">
+        <v>9</v>
+      </c>
+      <c r="E546" t="n">
+        <v>0</v>
+      </c>
+      <c r="F546" t="n">
+        <v>0</v>
+      </c>
+      <c r="G546" t="n">
+        <v>11001</v>
+      </c>
+      <c r="H546" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="547">
+      <c r="A547" t="n">
+        <v>544</v>
+      </c>
+      <c r="B547" t="n">
+        <v>30061</v>
+      </c>
+      <c r="C547" t="n">
+        <v>4</v>
+      </c>
+      <c r="D547" t="n">
+        <v>9</v>
+      </c>
+      <c r="E547" t="n">
+        <v>0</v>
+      </c>
+      <c r="F547" t="n">
+        <v>0</v>
+      </c>
+      <c r="G547" t="n">
+        <v>11001</v>
+      </c>
+      <c r="H547" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="548">
+      <c r="A548" t="n">
+        <v>545</v>
+      </c>
+      <c r="B548" t="n">
+        <v>30061</v>
+      </c>
+      <c r="C548" t="n">
+        <v>5</v>
+      </c>
+      <c r="D548" t="n">
+        <v>9</v>
+      </c>
+      <c r="E548" t="n">
+        <v>0</v>
+      </c>
+      <c r="F548" t="n">
+        <v>0</v>
+      </c>
+      <c r="G548" t="n">
+        <v>11001</v>
+      </c>
+      <c r="H548" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="549">
+      <c r="A549" t="n">
+        <v>546</v>
+      </c>
+      <c r="B549" t="n">
+        <v>30061</v>
+      </c>
+      <c r="C549" t="n">
+        <v>6</v>
+      </c>
+      <c r="D549" t="n">
+        <v>9</v>
+      </c>
+      <c r="E549" t="n">
+        <v>0</v>
+      </c>
+      <c r="F549" t="n">
+        <v>0</v>
+      </c>
+      <c r="G549" t="n">
+        <v>11001</v>
+      </c>
+      <c r="H549" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="550">
+      <c r="A550" t="n">
+        <v>547</v>
+      </c>
+      <c r="B550" t="n">
+        <v>30061</v>
+      </c>
+      <c r="C550" t="n">
+        <v>7</v>
+      </c>
+      <c r="D550" t="n">
+        <v>9</v>
+      </c>
+      <c r="E550" t="n">
+        <v>0</v>
+      </c>
+      <c r="F550" t="n">
+        <v>0</v>
+      </c>
+      <c r="G550" t="n">
+        <v>11001</v>
+      </c>
+      <c r="H550" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="551">
+      <c r="A551" t="n">
+        <v>548</v>
+      </c>
+      <c r="B551" t="n">
+        <v>30061</v>
+      </c>
+      <c r="C551" t="n">
+        <v>8</v>
+      </c>
+      <c r="D551" t="n">
+        <v>9</v>
+      </c>
+      <c r="E551" t="n">
+        <v>0</v>
+      </c>
+      <c r="F551" t="n">
+        <v>0</v>
+      </c>
+      <c r="G551" t="n">
+        <v>11001</v>
+      </c>
+      <c r="H551" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="552">
+      <c r="A552" t="n">
+        <v>549</v>
+      </c>
+      <c r="B552" t="n">
+        <v>30061</v>
+      </c>
+      <c r="C552" t="n">
+        <v>9</v>
+      </c>
+      <c r="D552" t="n">
+        <v>9</v>
+      </c>
+      <c r="E552" t="n">
+        <v>0</v>
+      </c>
+      <c r="F552" t="n">
+        <v>0</v>
+      </c>
+      <c r="G552" t="n">
+        <v>11001</v>
+      </c>
+      <c r="H552" t="n">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="553">
+      <c r="A553" t="n">
+        <v>550</v>
+      </c>
+      <c r="B553" t="n">
+        <v>30062</v>
+      </c>
+      <c r="C553" t="n">
+        <v>1</v>
+      </c>
+      <c r="D553" t="n">
+        <v>7</v>
+      </c>
+      <c r="E553" t="n">
+        <v>0</v>
+      </c>
+      <c r="F553" t="n">
+        <v>0</v>
+      </c>
+      <c r="G553" t="n">
+        <v>11001</v>
+      </c>
+      <c r="H553" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="554">
+      <c r="A554" t="n">
+        <v>551</v>
+      </c>
+      <c r="B554" t="n">
+        <v>30062</v>
+      </c>
+      <c r="C554" t="n">
+        <v>2</v>
+      </c>
+      <c r="D554" t="n">
+        <v>7</v>
+      </c>
+      <c r="E554" t="n">
+        <v>0</v>
+      </c>
+      <c r="F554" t="n">
+        <v>0</v>
+      </c>
+      <c r="G554" t="n">
+        <v>11001</v>
+      </c>
+      <c r="H554" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="555">
+      <c r="A555" t="n">
+        <v>552</v>
+      </c>
+      <c r="B555" t="n">
+        <v>30062</v>
+      </c>
+      <c r="C555" t="n">
+        <v>3</v>
+      </c>
+      <c r="D555" t="n">
+        <v>7</v>
+      </c>
+      <c r="E555" t="n">
+        <v>0</v>
+      </c>
+      <c r="F555" t="n">
+        <v>0</v>
+      </c>
+      <c r="G555" t="n">
+        <v>11001</v>
+      </c>
+      <c r="H555" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="556">
+      <c r="A556" t="n">
+        <v>553</v>
+      </c>
+      <c r="B556" t="n">
+        <v>30062</v>
+      </c>
+      <c r="C556" t="n">
+        <v>4</v>
+      </c>
+      <c r="D556" t="n">
+        <v>7</v>
+      </c>
+      <c r="E556" t="n">
+        <v>0</v>
+      </c>
+      <c r="F556" t="n">
+        <v>0</v>
+      </c>
+      <c r="G556" t="n">
+        <v>11001</v>
+      </c>
+      <c r="H556" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="557">
+      <c r="A557" t="n">
+        <v>554</v>
+      </c>
+      <c r="B557" t="n">
+        <v>30062</v>
+      </c>
+      <c r="C557" t="n">
+        <v>5</v>
+      </c>
+      <c r="D557" t="n">
+        <v>7</v>
+      </c>
+      <c r="E557" t="n">
+        <v>0</v>
+      </c>
+      <c r="F557" t="n">
+        <v>0</v>
+      </c>
+      <c r="G557" t="n">
+        <v>11001</v>
+      </c>
+      <c r="H557" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="558">
+      <c r="A558" t="n">
+        <v>555</v>
+      </c>
+      <c r="B558" t="n">
+        <v>30062</v>
+      </c>
+      <c r="C558" t="n">
+        <v>6</v>
+      </c>
+      <c r="D558" t="n">
+        <v>7</v>
+      </c>
+      <c r="E558" t="n">
+        <v>0</v>
+      </c>
+      <c r="F558" t="n">
+        <v>0</v>
+      </c>
+      <c r="G558" t="n">
+        <v>11001</v>
+      </c>
+      <c r="H558" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="559">
+      <c r="A559" t="n">
+        <v>556</v>
+      </c>
+      <c r="B559" t="n">
+        <v>30062</v>
+      </c>
+      <c r="C559" t="n">
+        <v>7</v>
+      </c>
+      <c r="D559" t="n">
+        <v>7</v>
+      </c>
+      <c r="E559" t="n">
+        <v>0</v>
+      </c>
+      <c r="F559" t="n">
+        <v>0</v>
+      </c>
+      <c r="G559" t="n">
+        <v>11001</v>
+      </c>
+      <c r="H559" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="560">
+      <c r="A560" t="n">
+        <v>557</v>
+      </c>
+      <c r="B560" t="n">
+        <v>30062</v>
+      </c>
+      <c r="C560" t="n">
+        <v>8</v>
+      </c>
+      <c r="D560" t="n">
+        <v>7</v>
+      </c>
+      <c r="E560" t="n">
+        <v>0</v>
+      </c>
+      <c r="F560" t="n">
+        <v>0</v>
+      </c>
+      <c r="G560" t="n">
+        <v>11001</v>
+      </c>
+      <c r="H560" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="561">
+      <c r="A561" t="n">
+        <v>558</v>
+      </c>
+      <c r="B561" t="n">
+        <v>30062</v>
+      </c>
+      <c r="C561" t="n">
+        <v>9</v>
+      </c>
+      <c r="D561" t="n">
+        <v>7</v>
+      </c>
+      <c r="E561" t="n">
+        <v>0</v>
+      </c>
+      <c r="F561" t="n">
+        <v>0</v>
+      </c>
+      <c r="G561" t="n">
+        <v>11001</v>
+      </c>
+      <c r="H561" t="n">
+        <v>27</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>